<commit_message>
header was missing in "total" column
</commit_message>
<xml_diff>
--- a/data/compiling/2025/CRSR/Junquillal/Santa_Rosa_lista_aves_actualizada_2026 Junquillal Norte.xlsx
+++ b/data/compiling/2025/CRSR/Junquillal/Santa_Rosa_lista_aves_actualizada_2026 Junquillal Norte.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10222"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CRIST\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisjoyce/GitHub/CBC/ACG-CBC-data/data/compiling/2025/CRSR/Junquillal/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF1DB0B-8E40-2B46-999C-C9F3A6BEC1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="12340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRSR_2023_updated_cleaned" sheetId="1" r:id="rId1"/>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="948">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="949">
   <si>
     <t>Familia</t>
   </si>
@@ -2867,12 +2868,15 @@
   </si>
   <si>
     <t>Saucerottia hoffmanni</t>
+  </si>
+  <si>
+    <t>total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -3391,48 +3395,48 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3743,19 +3747,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F363"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.375" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.5" style="2" customWidth="1"/>
-    <col min="4" max="4" width="36.875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="5.375" customWidth="1"/>
-    <col min="6" max="6" width="15.875" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="5.33203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3768,12 +3772,14 @@
       <c r="D1" s="4" t="s">
         <v>945</v>
       </c>
-      <c r="E1" s="3"/>
+      <c r="E1" s="3" t="s">
+        <v>948</v>
+      </c>
       <c r="F1" s="3" t="s">
         <v>943</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -3783,7 +3789,7 @@
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
       <c r="B3" s="7" t="s">
         <v>2</v>
@@ -3797,7 +3803,7 @@
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -3807,7 +3813,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="7" t="s">
         <v>6</v>
@@ -3821,7 +3827,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
       <c r="B6" s="7" t="s">
         <v>9</v>
@@ -3835,7 +3841,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="3"/>
       <c r="B7" s="7" t="s">
         <v>12</v>
@@ -3849,7 +3855,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
       <c r="B8" s="7" t="s">
         <v>15</v>
@@ -3863,7 +3869,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>18</v>
       </c>
@@ -3873,7 +3879,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
       <c r="B10" s="7" t="s">
         <v>19</v>
@@ -3887,7 +3893,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="7" t="s">
         <v>22</v>
@@ -3901,7 +3907,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="B12" s="7" t="s">
         <v>25</v>
@@ -3915,7 +3921,7 @@
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -3925,7 +3931,7 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="7" t="s">
         <v>29</v>
@@ -3939,7 +3945,7 @@
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>32</v>
       </c>
@@ -3949,7 +3955,7 @@
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="7" t="s">
         <v>33</v>
@@ -3963,7 +3969,7 @@
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>36</v>
       </c>
@@ -3973,7 +3979,7 @@
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" s="7" t="s">
         <v>37</v>
@@ -3987,7 +3993,7 @@
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="7" t="s">
         <v>40</v>
@@ -4001,7 +4007,7 @@
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="7" t="s">
         <v>43</v>
@@ -4015,7 +4021,7 @@
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="7" t="s">
         <v>46</v>
@@ -4029,7 +4035,7 @@
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
     </row>
-    <row r="22" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="7" t="s">
         <v>49</v>
@@ -4043,7 +4049,7 @@
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="7" t="s">
         <v>52</v>
@@ -4059,7 +4065,7 @@
       </c>
       <c r="F23" s="5"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
       <c r="B24" s="7" t="s">
         <v>55</v>
@@ -4073,7 +4079,7 @@
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
     </row>
-    <row r="25" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="B25" s="7" t="s">
         <v>58</v>
@@ -4087,7 +4093,7 @@
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
     </row>
-    <row r="26" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="7" t="s">
         <v>61</v>
@@ -4101,7 +4107,7 @@
       <c r="E26" s="5"/>
       <c r="F26" s="5"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="7" t="s">
         <v>64</v>
@@ -4115,7 +4121,7 @@
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="7" t="s">
         <v>67</v>
@@ -4131,7 +4137,7 @@
       </c>
       <c r="F28" s="5"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="B29" s="7" t="s">
         <v>70</v>
@@ -4145,7 +4151,7 @@
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="7" t="s">
         <v>73</v>
@@ -4159,7 +4165,7 @@
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
       <c r="B31" s="7" t="s">
         <v>76</v>
@@ -4175,7 +4181,7 @@
       </c>
       <c r="F31" s="5"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
       <c r="B32" s="7" t="s">
         <v>79</v>
@@ -4189,7 +4195,7 @@
       <c r="E32" s="5"/>
       <c r="F32" s="5"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>82</v>
       </c>
@@ -4199,7 +4205,7 @@
       <c r="E33" s="5"/>
       <c r="F33" s="5"/>
     </row>
-    <row r="34" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A34" s="3"/>
       <c r="B34" s="7" t="s">
         <v>83</v>
@@ -4213,7 +4219,7 @@
       <c r="E34" s="5"/>
       <c r="F34" s="5"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="7" t="s">
         <v>86</v>
@@ -4227,7 +4233,7 @@
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
     </row>
-    <row r="36" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
       <c r="B36" s="7" t="s">
         <v>89</v>
@@ -4241,7 +4247,7 @@
       <c r="E36" s="5"/>
       <c r="F36" s="5"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
       <c r="B37" s="7" t="s">
         <v>92</v>
@@ -4255,7 +4261,7 @@
       <c r="E37" s="5"/>
       <c r="F37" s="5"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>95</v>
       </c>
@@ -4265,7 +4271,7 @@
       <c r="E38" s="5"/>
       <c r="F38" s="5"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
       <c r="B39" s="7" t="s">
         <v>96</v>
@@ -4281,7 +4287,7 @@
       </c>
       <c r="F39" s="5"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
       <c r="B40" s="7" t="s">
         <v>99</v>
@@ -4295,7 +4301,7 @@
       <c r="E40" s="5"/>
       <c r="F40" s="5"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
       <c r="B41" s="7" t="s">
         <v>102</v>
@@ -4309,7 +4315,7 @@
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="3"/>
       <c r="B42" s="7" t="s">
         <v>105</v>
@@ -4323,7 +4329,7 @@
       <c r="E42" s="5"/>
       <c r="F42" s="5"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>108</v>
       </c>
@@ -4333,7 +4339,7 @@
       <c r="E43" s="5"/>
       <c r="F43" s="5"/>
     </row>
-    <row r="44" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="7" t="s">
         <v>109</v>
@@ -4347,7 +4353,7 @@
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="3"/>
       <c r="B45" s="7" t="s">
         <v>112</v>
@@ -4361,7 +4367,7 @@
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>115</v>
       </c>
@@ -4371,7 +4377,7 @@
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="3"/>
       <c r="B47" s="7" t="s">
         <v>116</v>
@@ -4385,7 +4391,7 @@
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="3"/>
       <c r="B48" s="7" t="s">
         <v>119</v>
@@ -4399,7 +4405,7 @@
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>122</v>
       </c>
@@ -4409,7 +4415,7 @@
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="3"/>
       <c r="B50" s="7" t="s">
         <v>123</v>
@@ -4423,7 +4429,7 @@
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="3"/>
       <c r="B51" s="7" t="s">
         <v>126</v>
@@ -4437,7 +4443,7 @@
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="3"/>
       <c r="B52" s="7" t="s">
         <v>129</v>
@@ -4451,7 +4457,7 @@
       <c r="E52" s="5"/>
       <c r="F52" s="5"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A53" s="3"/>
       <c r="B53" s="7" t="s">
         <v>132</v>
@@ -4465,7 +4471,7 @@
       <c r="E53" s="5"/>
       <c r="F53" s="5"/>
     </row>
-    <row r="54" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="3"/>
       <c r="B54" s="7" t="s">
         <v>135</v>
@@ -4479,7 +4485,7 @@
       <c r="E54" s="5"/>
       <c r="F54" s="5"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="3"/>
       <c r="B55" s="7" t="s">
         <v>138</v>
@@ -4493,7 +4499,7 @@
       <c r="E55" s="5"/>
       <c r="F55" s="5"/>
     </row>
-    <row r="56" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="3"/>
       <c r="B56" s="7" t="s">
         <v>141</v>
@@ -4507,7 +4513,7 @@
       <c r="E56" s="5"/>
       <c r="F56" s="5"/>
     </row>
-    <row r="57" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A57" s="3"/>
       <c r="B57" s="7" t="s">
         <v>947</v>
@@ -4521,7 +4527,7 @@
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A58" s="3"/>
       <c r="B58" s="7" t="s">
         <v>145</v>
@@ -4537,7 +4543,7 @@
       </c>
       <c r="F58" s="5"/>
     </row>
-    <row r="59" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A59" s="3"/>
       <c r="B59" s="7" t="s">
         <v>148</v>
@@ -4551,7 +4557,7 @@
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
-    <row r="60" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A60" s="3"/>
       <c r="B60" s="7" t="s">
         <v>151</v>
@@ -4565,7 +4571,7 @@
       <c r="E60" s="5"/>
       <c r="F60" s="5"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>154</v>
       </c>
@@ -4575,7 +4581,7 @@
       <c r="E61" s="5"/>
       <c r="F61" s="5"/>
     </row>
-    <row r="62" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A62" s="3"/>
       <c r="B62" s="7" t="s">
         <v>155</v>
@@ -4589,7 +4595,7 @@
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
     </row>
-    <row r="63" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A63" s="3"/>
       <c r="B63" s="7" t="s">
         <v>158</v>
@@ -4605,7 +4611,7 @@
       </c>
       <c r="F63" s="5"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="3"/>
       <c r="B64" s="7" t="s">
         <v>161</v>
@@ -4619,7 +4625,7 @@
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="3"/>
       <c r="B65" s="7" t="s">
         <v>164</v>
@@ -4633,7 +4639,7 @@
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
     </row>
-    <row r="66" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" s="3"/>
       <c r="B66" s="7" t="s">
         <v>167</v>
@@ -4647,7 +4653,7 @@
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="3"/>
       <c r="B67" s="7" t="s">
         <v>170</v>
@@ -4661,7 +4667,7 @@
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>173</v>
       </c>
@@ -4671,7 +4677,7 @@
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="3"/>
       <c r="B69" s="7" t="s">
         <v>174</v>
@@ -4687,7 +4693,7 @@
       </c>
       <c r="F69" s="5"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
         <v>177</v>
       </c>
@@ -4697,7 +4703,7 @@
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
     </row>
-    <row r="71" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A71" s="3"/>
       <c r="B71" s="7" t="s">
         <v>178</v>
@@ -4711,7 +4717,7 @@
       <c r="E71" s="5"/>
       <c r="F71" s="5"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
         <v>181</v>
       </c>
@@ -4721,7 +4727,7 @@
       <c r="E72" s="5"/>
       <c r="F72" s="5"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="3"/>
       <c r="B73" s="7" t="s">
         <v>182</v>
@@ -4737,7 +4743,7 @@
       </c>
       <c r="F73" s="5"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>185</v>
       </c>
@@ -4747,7 +4753,7 @@
       <c r="E74" s="5"/>
       <c r="F74" s="5"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" s="3"/>
       <c r="B75" s="7" t="s">
         <v>186</v>
@@ -4761,7 +4767,7 @@
       <c r="E75" s="5"/>
       <c r="F75" s="5"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
         <v>189</v>
       </c>
@@ -4771,7 +4777,7 @@
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="3"/>
       <c r="B77" s="7" t="s">
         <v>190</v>
@@ -4785,7 +4791,7 @@
       <c r="E77" s="5"/>
       <c r="F77" s="5"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A78" s="3"/>
       <c r="B78" s="7" t="s">
         <v>193</v>
@@ -4799,7 +4805,7 @@
       <c r="E78" s="5"/>
       <c r="F78" s="5"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A79" s="3"/>
       <c r="B79" s="7" t="s">
         <v>196</v>
@@ -4813,7 +4819,7 @@
       <c r="E79" s="5"/>
       <c r="F79" s="5"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A80" s="3"/>
       <c r="B80" s="7" t="s">
         <v>199</v>
@@ -4827,7 +4833,7 @@
       <c r="E80" s="5"/>
       <c r="F80" s="5"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A81" s="3"/>
       <c r="B81" s="7" t="s">
         <v>202</v>
@@ -4841,7 +4847,7 @@
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A82" s="3"/>
       <c r="B82" s="7" t="s">
         <v>205</v>
@@ -4855,7 +4861,7 @@
       <c r="E82" s="5"/>
       <c r="F82" s="5"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A83" s="3"/>
       <c r="B83" s="7" t="s">
         <v>208</v>
@@ -4869,7 +4875,7 @@
       <c r="E83" s="5"/>
       <c r="F83" s="5"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
         <v>211</v>
       </c>
@@ -4879,7 +4885,7 @@
       <c r="E84" s="5"/>
       <c r="F84" s="5"/>
     </row>
-    <row r="85" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A85" s="3"/>
       <c r="B85" s="7" t="s">
         <v>212</v>
@@ -4893,7 +4899,7 @@
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
         <v>215</v>
       </c>
@@ -4903,7 +4909,7 @@
       <c r="E86" s="5"/>
       <c r="F86" s="5"/>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="3"/>
       <c r="B87" s="7" t="s">
         <v>216</v>
@@ -4919,7 +4925,7 @@
       </c>
       <c r="F87" s="5"/>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" s="3"/>
       <c r="B88" s="7" t="s">
         <v>219</v>
@@ -4933,7 +4939,7 @@
       <c r="E88" s="5"/>
       <c r="F88" s="5"/>
     </row>
-    <row r="89" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A89" s="3"/>
       <c r="B89" s="7" t="s">
         <v>222</v>
@@ -4949,7 +4955,7 @@
       </c>
       <c r="F89" s="5"/>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A90" s="3"/>
       <c r="B90" s="7" t="s">
         <v>225</v>
@@ -4965,7 +4971,7 @@
       </c>
       <c r="F90" s="5"/>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A91" s="3"/>
       <c r="B91" s="7" t="s">
         <v>228</v>
@@ -4981,7 +4987,7 @@
       </c>
       <c r="F91" s="5"/>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A92" s="3"/>
       <c r="B92" s="7" t="s">
         <v>231</v>
@@ -4997,7 +5003,7 @@
       </c>
       <c r="F92" s="5"/>
     </row>
-    <row r="93" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A93" s="3"/>
       <c r="B93" s="7" t="s">
         <v>234</v>
@@ -5011,7 +5017,7 @@
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A94" s="3"/>
       <c r="B94" s="7" t="s">
         <v>237</v>
@@ -5025,7 +5031,7 @@
       <c r="E94" s="5"/>
       <c r="F94" s="5"/>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A95" s="3"/>
       <c r="B95" s="7" t="s">
         <v>240</v>
@@ -5039,7 +5045,7 @@
       <c r="E95" s="5"/>
       <c r="F95" s="5"/>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A96" s="3"/>
       <c r="B96" s="7" t="s">
         <v>243</v>
@@ -5055,7 +5061,7 @@
       </c>
       <c r="F96" s="5"/>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A97" s="3"/>
       <c r="B97" s="7" t="s">
         <v>246</v>
@@ -5071,7 +5077,7 @@
       </c>
       <c r="F97" s="5"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A98" s="3"/>
       <c r="B98" s="7" t="s">
         <v>249</v>
@@ -5087,7 +5093,7 @@
       </c>
       <c r="F98" s="5"/>
     </row>
-    <row r="99" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A99" s="3"/>
       <c r="B99" s="7" t="s">
         <v>252</v>
@@ -5101,7 +5107,7 @@
       <c r="E99" s="5"/>
       <c r="F99" s="5"/>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
         <v>255</v>
       </c>
@@ -5111,7 +5117,7 @@
       <c r="E100" s="5"/>
       <c r="F100" s="5"/>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A101" s="3"/>
       <c r="B101" s="7" t="s">
         <v>256</v>
@@ -5125,7 +5131,7 @@
       <c r="E101" s="5"/>
       <c r="F101" s="5"/>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" s="3"/>
       <c r="B102" s="7" t="s">
         <v>259</v>
@@ -5141,7 +5147,7 @@
       </c>
       <c r="F102" s="5"/>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A103" s="3"/>
       <c r="B103" s="7" t="s">
         <v>262</v>
@@ -5155,7 +5161,7 @@
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A104" s="3"/>
       <c r="B104" s="7" t="s">
         <v>265</v>
@@ -5169,7 +5175,7 @@
       <c r="E104" s="5"/>
       <c r="F104" s="5"/>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A105" s="3"/>
       <c r="B105" s="7" t="s">
         <v>268</v>
@@ -5183,7 +5189,7 @@
       <c r="E105" s="5"/>
       <c r="F105" s="5"/>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A106" s="3"/>
       <c r="B106" s="7" t="s">
         <v>271</v>
@@ -5197,7 +5203,7 @@
       <c r="E106" s="5"/>
       <c r="F106" s="5"/>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A107" s="3"/>
       <c r="B107" s="7" t="s">
         <v>274</v>
@@ -5213,7 +5219,7 @@
       </c>
       <c r="F107" s="5"/>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="s">
         <v>277</v>
       </c>
@@ -5223,7 +5229,7 @@
       <c r="E108" s="5"/>
       <c r="F108" s="5"/>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A109" s="3"/>
       <c r="B109" s="7" t="s">
         <v>278</v>
@@ -5237,7 +5243,7 @@
       <c r="E109" s="5"/>
       <c r="F109" s="5"/>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="3" t="s">
         <v>281</v>
       </c>
@@ -5247,7 +5253,7 @@
       <c r="E110" s="5"/>
       <c r="F110" s="5"/>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A111" s="3"/>
       <c r="B111" s="7" t="s">
         <v>282</v>
@@ -5263,7 +5269,7 @@
       </c>
       <c r="F111" s="5"/>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" s="3" t="s">
         <v>285</v>
       </c>
@@ -5273,7 +5279,7 @@
       <c r="E112" s="5"/>
       <c r="F112" s="5"/>
     </row>
-    <row r="113" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A113" s="3"/>
       <c r="B113" s="7" t="s">
         <v>286</v>
@@ -5289,7 +5295,7 @@
       </c>
       <c r="F113" s="5"/>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" s="3" t="s">
         <v>289</v>
       </c>
@@ -5299,7 +5305,7 @@
       <c r="E114" s="5"/>
       <c r="F114" s="5"/>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A115" s="3"/>
       <c r="B115" s="7" t="s">
         <v>290</v>
@@ -5313,7 +5319,7 @@
       <c r="E115" s="5"/>
       <c r="F115" s="5"/>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A116" s="3"/>
       <c r="B116" s="7" t="s">
         <v>293</v>
@@ -5327,7 +5333,7 @@
       <c r="E116" s="5"/>
       <c r="F116" s="5"/>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A117" s="3"/>
       <c r="B117" s="7" t="s">
         <v>296</v>
@@ -5341,7 +5347,7 @@
       <c r="E117" s="5"/>
       <c r="F117" s="5"/>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="3" t="s">
         <v>299</v>
       </c>
@@ -5351,7 +5357,7 @@
       <c r="E118" s="5"/>
       <c r="F118" s="5"/>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A119" s="3"/>
       <c r="B119" s="7" t="s">
         <v>300</v>
@@ -5365,7 +5371,7 @@
       <c r="E119" s="5"/>
       <c r="F119" s="5"/>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="3" t="s">
         <v>303</v>
       </c>
@@ -5375,7 +5381,7 @@
       <c r="E120" s="5"/>
       <c r="F120" s="5"/>
     </row>
-    <row r="121" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A121" s="3"/>
       <c r="B121" s="7" t="s">
         <v>304</v>
@@ -5389,7 +5395,7 @@
       <c r="E121" s="5"/>
       <c r="F121" s="5"/>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="3" t="s">
         <v>307</v>
       </c>
@@ -5399,7 +5405,7 @@
       <c r="E122" s="5"/>
       <c r="F122" s="5"/>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A123" s="3"/>
       <c r="B123" s="7" t="s">
         <v>308</v>
@@ -5415,7 +5421,7 @@
       </c>
       <c r="F123" s="5"/>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="3" t="s">
         <v>311</v>
       </c>
@@ -5425,7 +5431,7 @@
       <c r="E124" s="5"/>
       <c r="F124" s="5"/>
     </row>
-    <row r="125" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A125" s="3"/>
       <c r="B125" s="7" t="s">
         <v>312</v>
@@ -5441,7 +5447,7 @@
       </c>
       <c r="F125" s="5"/>
     </row>
-    <row r="126" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A126" s="3"/>
       <c r="B126" s="7" t="s">
         <v>315</v>
@@ -5455,7 +5461,7 @@
       <c r="E126" s="5"/>
       <c r="F126" s="5"/>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A127" s="3"/>
       <c r="B127" s="7" t="s">
         <v>318</v>
@@ -5469,7 +5475,7 @@
       <c r="E127" s="5"/>
       <c r="F127" s="5"/>
     </row>
-    <row r="128" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A128" s="3"/>
       <c r="B128" s="7" t="s">
         <v>321</v>
@@ -5485,7 +5491,7 @@
       </c>
       <c r="F128" s="5"/>
     </row>
-    <row r="129" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A129" s="3"/>
       <c r="B129" s="7" t="s">
         <v>324</v>
@@ -5499,7 +5505,7 @@
       <c r="E129" s="5"/>
       <c r="F129" s="5"/>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A130" s="3"/>
       <c r="B130" s="7" t="s">
         <v>327</v>
@@ -5513,7 +5519,7 @@
       <c r="E130" s="5"/>
       <c r="F130" s="5"/>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A131" s="3"/>
       <c r="B131" s="7" t="s">
         <v>330</v>
@@ -5527,7 +5533,7 @@
       <c r="E131" s="5"/>
       <c r="F131" s="5"/>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A132" s="3"/>
       <c r="B132" s="7" t="s">
         <v>333</v>
@@ -5541,7 +5547,7 @@
       <c r="E132" s="5"/>
       <c r="F132" s="5"/>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A133" s="3"/>
       <c r="B133" s="7" t="s">
         <v>336</v>
@@ -5557,7 +5563,7 @@
       </c>
       <c r="F133" s="5"/>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A134" s="3"/>
       <c r="B134" s="7" t="s">
         <v>339</v>
@@ -5573,7 +5579,7 @@
       </c>
       <c r="F134" s="5"/>
     </row>
-    <row r="135" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A135" s="3"/>
       <c r="B135" s="7" t="s">
         <v>342</v>
@@ -5587,7 +5593,7 @@
       <c r="E135" s="5"/>
       <c r="F135" s="5"/>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A136" s="3"/>
       <c r="B136" s="7" t="s">
         <v>345</v>
@@ -5603,7 +5609,7 @@
       </c>
       <c r="F136" s="5"/>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A137" s="3"/>
       <c r="B137" s="7" t="s">
         <v>348</v>
@@ -5619,7 +5625,7 @@
       </c>
       <c r="F137" s="5"/>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" s="3" t="s">
         <v>351</v>
       </c>
@@ -5629,7 +5635,7 @@
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A139" s="3"/>
       <c r="B139" s="7" t="s">
         <v>352</v>
@@ -5645,7 +5651,7 @@
       </c>
       <c r="F139" s="5"/>
     </row>
-    <row r="140" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A140" s="3"/>
       <c r="B140" s="7" t="s">
         <v>355</v>
@@ -5661,7 +5667,7 @@
       </c>
       <c r="F140" s="5"/>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" s="3" t="s">
         <v>358</v>
       </c>
@@ -5671,7 +5677,7 @@
       <c r="E141" s="5"/>
       <c r="F141" s="5"/>
     </row>
-    <row r="142" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A142" s="3"/>
       <c r="B142" s="7" t="s">
         <v>359</v>
@@ -5685,7 +5691,7 @@
       <c r="E142" s="5"/>
       <c r="F142" s="5"/>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A143" s="3"/>
       <c r="B143" s="7" t="s">
         <v>362</v>
@@ -5701,7 +5707,7 @@
       </c>
       <c r="F143" s="5"/>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A144" s="3"/>
       <c r="B144" s="7" t="s">
         <v>365</v>
@@ -5717,7 +5723,7 @@
       </c>
       <c r="F144" s="5"/>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" s="3" t="s">
         <v>368</v>
       </c>
@@ -5727,7 +5733,7 @@
       <c r="E145" s="5"/>
       <c r="F145" s="5"/>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A146" s="3"/>
       <c r="B146" s="7" t="s">
         <v>369</v>
@@ -5741,7 +5747,7 @@
       <c r="E146" s="5"/>
       <c r="F146" s="5"/>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" s="3" t="s">
         <v>372</v>
       </c>
@@ -5751,7 +5757,7 @@
       <c r="E147" s="5"/>
       <c r="F147" s="5"/>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A148" s="3"/>
       <c r="B148" s="7" t="s">
         <v>373</v>
@@ -5765,7 +5771,7 @@
       <c r="E148" s="5"/>
       <c r="F148" s="5"/>
     </row>
-    <row r="149" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A149" s="3"/>
       <c r="B149" s="7" t="s">
         <v>376</v>
@@ -5779,7 +5785,7 @@
       <c r="E149" s="5"/>
       <c r="F149" s="5"/>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A150" s="3"/>
       <c r="B150" s="7" t="s">
         <v>379</v>
@@ -5793,7 +5799,7 @@
       <c r="E150" s="5"/>
       <c r="F150" s="5"/>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A151" s="3"/>
       <c r="B151" s="7" t="s">
         <v>382</v>
@@ -5807,7 +5813,7 @@
       <c r="E151" s="5"/>
       <c r="F151" s="5"/>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A152" s="3"/>
       <c r="B152" s="7" t="s">
         <v>385</v>
@@ -5821,7 +5827,7 @@
       <c r="E152" s="5"/>
       <c r="F152" s="5"/>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A153" s="3"/>
       <c r="B153" s="7" t="s">
         <v>388</v>
@@ -5835,7 +5841,7 @@
       <c r="E153" s="5"/>
       <c r="F153" s="5"/>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A154" s="3"/>
       <c r="B154" s="7" t="s">
         <v>391</v>
@@ -5849,7 +5855,7 @@
       <c r="E154" s="5"/>
       <c r="F154" s="5"/>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A155" s="3"/>
       <c r="B155" s="7" t="s">
         <v>394</v>
@@ -5863,7 +5869,7 @@
       <c r="E155" s="5"/>
       <c r="F155" s="5"/>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A156" s="3"/>
       <c r="B156" s="7" t="s">
         <v>397</v>
@@ -5877,7 +5883,7 @@
       <c r="E156" s="5"/>
       <c r="F156" s="5"/>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A157" s="3"/>
       <c r="B157" s="7" t="s">
         <v>400</v>
@@ -5893,7 +5899,7 @@
       </c>
       <c r="F157" s="5"/>
     </row>
-    <row r="158" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A158" s="3"/>
       <c r="B158" s="7" t="s">
         <v>403</v>
@@ -5907,7 +5913,7 @@
       <c r="E158" s="5"/>
       <c r="F158" s="5"/>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A159" s="3"/>
       <c r="B159" s="7" t="s">
         <v>406</v>
@@ -5923,7 +5929,7 @@
       </c>
       <c r="F159" s="5"/>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A160" s="3"/>
       <c r="B160" s="7" t="s">
         <v>409</v>
@@ -5937,7 +5943,7 @@
       <c r="E160" s="5"/>
       <c r="F160" s="5"/>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A161" s="3"/>
       <c r="B161" s="7" t="s">
         <v>412</v>
@@ -5953,7 +5959,7 @@
       </c>
       <c r="F161" s="5"/>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A162" s="3"/>
       <c r="B162" s="7" t="s">
         <v>415</v>
@@ -5967,7 +5973,7 @@
       <c r="E162" s="5"/>
       <c r="F162" s="5"/>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A163" s="3"/>
       <c r="B163" s="7" t="s">
         <v>418</v>
@@ -5983,7 +5989,7 @@
       </c>
       <c r="F163" s="5"/>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A164" s="3"/>
       <c r="B164" s="7" t="s">
         <v>421</v>
@@ -5997,7 +6003,7 @@
       <c r="E164" s="5"/>
       <c r="F164" s="5"/>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A165" s="3"/>
       <c r="B165" s="7" t="s">
         <v>424</v>
@@ -6011,7 +6017,7 @@
       <c r="E165" s="5"/>
       <c r="F165" s="5"/>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" s="3" t="s">
         <v>427</v>
       </c>
@@ -6021,7 +6027,7 @@
       <c r="E166" s="5"/>
       <c r="F166" s="5"/>
     </row>
-    <row r="167" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A167" s="3"/>
       <c r="B167" s="7" t="s">
         <v>428</v>
@@ -6035,7 +6041,7 @@
       <c r="E167" s="5"/>
       <c r="F167" s="5"/>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A168" s="3" t="s">
         <v>431</v>
       </c>
@@ -6045,7 +6051,7 @@
       <c r="E168" s="5"/>
       <c r="F168" s="5"/>
     </row>
-    <row r="169" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A169" s="3"/>
       <c r="B169" s="7" t="s">
         <v>432</v>
@@ -6059,7 +6065,7 @@
       <c r="E169" s="5"/>
       <c r="F169" s="5"/>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A170" s="3"/>
       <c r="B170" s="7" t="s">
         <v>435</v>
@@ -6073,7 +6079,7 @@
       <c r="E170" s="5"/>
       <c r="F170" s="5"/>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A171" s="3"/>
       <c r="B171" s="7" t="s">
         <v>438</v>
@@ -6087,7 +6093,7 @@
       <c r="E171" s="5"/>
       <c r="F171" s="5"/>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A172" s="3"/>
       <c r="B172" s="7" t="s">
         <v>441</v>
@@ -6101,7 +6107,7 @@
       <c r="E172" s="5"/>
       <c r="F172" s="5"/>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" s="3" t="s">
         <v>444</v>
       </c>
@@ -6111,7 +6117,7 @@
       <c r="E173" s="5"/>
       <c r="F173" s="5"/>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A174" s="3"/>
       <c r="B174" s="7" t="s">
         <v>445</v>
@@ -6127,7 +6133,7 @@
       </c>
       <c r="F174" s="5"/>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A175" s="3"/>
       <c r="B175" s="7" t="s">
         <v>448</v>
@@ -6143,7 +6149,7 @@
       </c>
       <c r="F175" s="5"/>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A176" s="3"/>
       <c r="B176" s="7" t="s">
         <v>451</v>
@@ -6157,7 +6163,7 @@
       <c r="E176" s="5"/>
       <c r="F176" s="5"/>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A177" s="3" t="s">
         <v>454</v>
       </c>
@@ -6167,7 +6173,7 @@
       <c r="E177" s="5"/>
       <c r="F177" s="5"/>
     </row>
-    <row r="178" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A178" s="3"/>
       <c r="B178" s="7" t="s">
         <v>455</v>
@@ -6181,7 +6187,7 @@
       <c r="E178" s="5"/>
       <c r="F178" s="5"/>
     </row>
-    <row r="179" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A179" s="3"/>
       <c r="B179" s="7" t="s">
         <v>458</v>
@@ -6195,7 +6201,7 @@
       <c r="E179" s="5"/>
       <c r="F179" s="5"/>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A180" s="3" t="s">
         <v>461</v>
       </c>
@@ -6205,7 +6211,7 @@
       <c r="E180" s="5"/>
       <c r="F180" s="5"/>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A181" s="3"/>
       <c r="B181" s="7" t="s">
         <v>462</v>
@@ -6221,7 +6227,7 @@
       </c>
       <c r="F181" s="5"/>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A182" s="3"/>
       <c r="B182" s="7" t="s">
         <v>465</v>
@@ -6237,7 +6243,7 @@
       </c>
       <c r="F182" s="5"/>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A183" s="3"/>
       <c r="B183" s="7" t="s">
         <v>468</v>
@@ -6251,7 +6257,7 @@
       <c r="E183" s="5"/>
       <c r="F183" s="5"/>
     </row>
-    <row r="184" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A184" s="3"/>
       <c r="B184" s="7" t="s">
         <v>471</v>
@@ -6265,7 +6271,7 @@
       <c r="E184" s="5"/>
       <c r="F184" s="5"/>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A185" s="3"/>
       <c r="B185" s="7" t="s">
         <v>474</v>
@@ -6281,7 +6287,7 @@
       </c>
       <c r="F185" s="5"/>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A186" s="3" t="s">
         <v>477</v>
       </c>
@@ -6291,7 +6297,7 @@
       <c r="E186" s="5"/>
       <c r="F186" s="5"/>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A187" s="3"/>
       <c r="B187" s="7" t="s">
         <v>478</v>
@@ -6305,7 +6311,7 @@
       <c r="E187" s="5"/>
       <c r="F187" s="5"/>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A188" s="3" t="s">
         <v>481</v>
       </c>
@@ -6315,7 +6321,7 @@
       <c r="E188" s="5"/>
       <c r="F188" s="5"/>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A189" s="3"/>
       <c r="B189" s="7" t="s">
         <v>482</v>
@@ -6329,7 +6335,7 @@
       <c r="E189" s="5"/>
       <c r="F189" s="5"/>
     </row>
-    <row r="190" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A190" s="3"/>
       <c r="B190" s="7" t="s">
         <v>485</v>
@@ -6343,7 +6349,7 @@
       <c r="E190" s="5"/>
       <c r="F190" s="5"/>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A191" s="3" t="s">
         <v>488</v>
       </c>
@@ -6353,7 +6359,7 @@
       <c r="E191" s="5"/>
       <c r="F191" s="5"/>
     </row>
-    <row r="192" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A192" s="3"/>
       <c r="B192" s="7" t="s">
         <v>489</v>
@@ -6367,7 +6373,7 @@
       <c r="E192" s="5"/>
       <c r="F192" s="5"/>
     </row>
-    <row r="193" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A193" s="3"/>
       <c r="B193" s="7" t="s">
         <v>492</v>
@@ -6383,7 +6389,7 @@
       </c>
       <c r="F193" s="5"/>
     </row>
-    <row r="194" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A194" s="3"/>
       <c r="B194" s="7" t="s">
         <v>495</v>
@@ -6397,7 +6403,7 @@
       <c r="E194" s="5"/>
       <c r="F194" s="5"/>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A195" s="3"/>
       <c r="B195" s="7" t="s">
         <v>498</v>
@@ -6411,7 +6417,7 @@
       <c r="E195" s="5"/>
       <c r="F195" s="5"/>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A196" s="3" t="s">
         <v>501</v>
       </c>
@@ -6421,7 +6427,7 @@
       <c r="E196" s="5"/>
       <c r="F196" s="5"/>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A197" s="3"/>
       <c r="B197" s="7" t="s">
         <v>502</v>
@@ -6435,7 +6441,7 @@
       <c r="E197" s="5"/>
       <c r="F197" s="5"/>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A198" s="3"/>
       <c r="B198" s="7" t="s">
         <v>505</v>
@@ -6449,7 +6455,7 @@
       <c r="E198" s="5"/>
       <c r="F198" s="5"/>
     </row>
-    <row r="199" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A199" s="3"/>
       <c r="B199" s="7" t="s">
         <v>508</v>
@@ -6463,7 +6469,7 @@
       <c r="E199" s="5"/>
       <c r="F199" s="5"/>
     </row>
-    <row r="200" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A200" s="3"/>
       <c r="B200" s="7" t="s">
         <v>511</v>
@@ -6477,7 +6483,7 @@
       <c r="E200" s="5"/>
       <c r="F200" s="5"/>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A201" s="3"/>
       <c r="B201" s="7" t="s">
         <v>514</v>
@@ -6491,7 +6497,7 @@
       <c r="E201" s="5"/>
       <c r="F201" s="5"/>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A202" s="3"/>
       <c r="B202" s="7" t="s">
         <v>517</v>
@@ -6505,7 +6511,7 @@
       <c r="E202" s="5"/>
       <c r="F202" s="5"/>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A203" s="3"/>
       <c r="B203" s="7" t="s">
         <v>520</v>
@@ -6519,7 +6525,7 @@
       <c r="E203" s="5"/>
       <c r="F203" s="5"/>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A204" s="3"/>
       <c r="B204" s="7" t="s">
         <v>523</v>
@@ -6533,7 +6539,7 @@
       <c r="E204" s="5"/>
       <c r="F204" s="5"/>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A205" s="3" t="s">
         <v>526</v>
       </c>
@@ -6543,7 +6549,7 @@
       <c r="E205" s="5"/>
       <c r="F205" s="5"/>
     </row>
-    <row r="206" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A206" s="3"/>
       <c r="B206" s="7" t="s">
         <v>527</v>
@@ -6559,7 +6565,7 @@
       </c>
       <c r="F206" s="5"/>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A207" s="3"/>
       <c r="B207" s="7" t="s">
         <v>530</v>
@@ -6573,7 +6579,7 @@
       <c r="E207" s="5"/>
       <c r="F207" s="5"/>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A208" s="3"/>
       <c r="B208" s="7" t="s">
         <v>533</v>
@@ -6587,7 +6593,7 @@
       <c r="E208" s="5"/>
       <c r="F208" s="5"/>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A209" s="3"/>
       <c r="B209" s="7" t="s">
         <v>536</v>
@@ -6601,7 +6607,7 @@
       <c r="E209" s="5"/>
       <c r="F209" s="5"/>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A210" s="3"/>
       <c r="B210" s="7" t="s">
         <v>539</v>
@@ -6617,7 +6623,7 @@
       </c>
       <c r="F210" s="5"/>
     </row>
-    <row r="211" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A211" s="3"/>
       <c r="B211" s="7" t="s">
         <v>542</v>
@@ -6631,7 +6637,7 @@
       <c r="E211" s="5"/>
       <c r="F211" s="5"/>
     </row>
-    <row r="212" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A212" s="3"/>
       <c r="B212" s="7" t="s">
         <v>545</v>
@@ -6647,7 +6653,7 @@
       </c>
       <c r="F212" s="5"/>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A213" s="3" t="s">
         <v>548</v>
       </c>
@@ -6657,7 +6663,7 @@
       <c r="E213" s="5"/>
       <c r="F213" s="5"/>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A214" s="3"/>
       <c r="B214" s="7" t="s">
         <v>549</v>
@@ -6671,7 +6677,7 @@
       <c r="E214" s="5"/>
       <c r="F214" s="5"/>
     </row>
-    <row r="215" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A215" s="3"/>
       <c r="B215" s="7" t="s">
         <v>552</v>
@@ -6685,7 +6691,7 @@
       <c r="E215" s="5"/>
       <c r="F215" s="5"/>
     </row>
-    <row r="216" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A216" s="3"/>
       <c r="B216" s="7" t="s">
         <v>552</v>
@@ -6699,7 +6705,7 @@
       <c r="E216" s="5"/>
       <c r="F216" s="5"/>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A217" s="3" t="s">
         <v>555</v>
       </c>
@@ -6709,7 +6715,7 @@
       <c r="E217" s="5"/>
       <c r="F217" s="5"/>
     </row>
-    <row r="218" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A218" s="3"/>
       <c r="B218" s="7" t="s">
         <v>556</v>
@@ -6723,7 +6729,7 @@
       <c r="E218" s="5"/>
       <c r="F218" s="5"/>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A219" s="3"/>
       <c r="B219" s="7" t="s">
         <v>559</v>
@@ -6737,7 +6743,7 @@
       <c r="E219" s="5"/>
       <c r="F219" s="5"/>
     </row>
-    <row r="220" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A220" s="3"/>
       <c r="B220" s="7" t="s">
         <v>562</v>
@@ -6751,7 +6757,7 @@
       <c r="E220" s="5"/>
       <c r="F220" s="5"/>
     </row>
-    <row r="221" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A221" s="3"/>
       <c r="B221" s="7" t="s">
         <v>565</v>
@@ -6765,7 +6771,7 @@
       <c r="E221" s="5"/>
       <c r="F221" s="5"/>
     </row>
-    <row r="222" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A222" s="3"/>
       <c r="B222" s="7" t="s">
         <v>568</v>
@@ -6779,7 +6785,7 @@
       <c r="E222" s="5"/>
       <c r="F222" s="5"/>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A223" s="3"/>
       <c r="B223" s="7" t="s">
         <v>571</v>
@@ -6793,7 +6799,7 @@
       <c r="E223" s="5"/>
       <c r="F223" s="5"/>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A224" s="3" t="s">
         <v>574</v>
       </c>
@@ -6803,7 +6809,7 @@
       <c r="E224" s="5"/>
       <c r="F224" s="5"/>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A225" s="3"/>
       <c r="B225" s="7" t="s">
         <v>575</v>
@@ -6817,7 +6823,7 @@
       <c r="E225" s="5"/>
       <c r="F225" s="5"/>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A226" s="3" t="s">
         <v>578</v>
       </c>
@@ -6827,7 +6833,7 @@
       <c r="E226" s="5"/>
       <c r="F226" s="5"/>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A227" s="3"/>
       <c r="B227" s="7" t="s">
         <v>579</v>
@@ -6841,7 +6847,7 @@
       <c r="E227" s="5"/>
       <c r="F227" s="5"/>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A228" s="3"/>
       <c r="B228" s="7" t="s">
         <v>582</v>
@@ -6855,7 +6861,7 @@
       <c r="E228" s="5"/>
       <c r="F228" s="5"/>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A229" s="3"/>
       <c r="B229" s="7" t="s">
         <v>585</v>
@@ -6869,7 +6875,7 @@
       <c r="E229" s="5"/>
       <c r="F229" s="5"/>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A230" s="3"/>
       <c r="B230" s="7" t="s">
         <v>588</v>
@@ -6883,7 +6889,7 @@
       <c r="E230" s="5"/>
       <c r="F230" s="5"/>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A231" s="3" t="s">
         <v>591</v>
       </c>
@@ -6893,7 +6899,7 @@
       <c r="E231" s="5"/>
       <c r="F231" s="5"/>
     </row>
-    <row r="232" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A232" s="3"/>
       <c r="B232" s="7" t="s">
         <v>592</v>
@@ -6907,7 +6913,7 @@
       <c r="E232" s="5"/>
       <c r="F232" s="5"/>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A233" s="3" t="s">
         <v>595</v>
       </c>
@@ -6917,7 +6923,7 @@
       <c r="E233" s="5"/>
       <c r="F233" s="5"/>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A234" s="3"/>
       <c r="B234" s="7" t="s">
         <v>596</v>
@@ -6931,7 +6937,7 @@
       <c r="E234" s="5"/>
       <c r="F234" s="5"/>
     </row>
-    <row r="235" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A235" s="3"/>
       <c r="B235" s="7" t="s">
         <v>599</v>
@@ -6945,7 +6951,7 @@
       <c r="E235" s="5"/>
       <c r="F235" s="5"/>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A236" s="3"/>
       <c r="B236" s="7" t="s">
         <v>602</v>
@@ -6959,7 +6965,7 @@
       <c r="E236" s="5"/>
       <c r="F236" s="5"/>
     </row>
-    <row r="237" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A237" s="3"/>
       <c r="B237" s="7" t="s">
         <v>605</v>
@@ -6973,7 +6979,7 @@
       <c r="E237" s="5"/>
       <c r="F237" s="5"/>
     </row>
-    <row r="238" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A238" s="3"/>
       <c r="B238" s="7" t="s">
         <v>608</v>
@@ -6987,7 +6993,7 @@
       <c r="E238" s="5"/>
       <c r="F238" s="5"/>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A239" s="3"/>
       <c r="B239" s="7" t="s">
         <v>611</v>
@@ -7001,7 +7007,7 @@
       <c r="E239" s="5"/>
       <c r="F239" s="5"/>
     </row>
-    <row r="240" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A240" s="3"/>
       <c r="B240" s="7" t="s">
         <v>614</v>
@@ -7015,7 +7021,7 @@
       <c r="E240" s="5"/>
       <c r="F240" s="5"/>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A241" s="3"/>
       <c r="B241" s="7" t="s">
         <v>617</v>
@@ -7029,7 +7035,7 @@
       <c r="E241" s="5"/>
       <c r="F241" s="5"/>
     </row>
-    <row r="242" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A242" s="3"/>
       <c r="B242" s="7" t="s">
         <v>620</v>
@@ -7043,7 +7049,7 @@
       <c r="E242" s="5"/>
       <c r="F242" s="5"/>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A243" s="3"/>
       <c r="B243" s="7" t="s">
         <v>623</v>
@@ -7057,7 +7063,7 @@
       <c r="E243" s="5"/>
       <c r="F243" s="5"/>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A244" s="3"/>
       <c r="B244" s="7" t="s">
         <v>626</v>
@@ -7071,7 +7077,7 @@
       <c r="E244" s="5"/>
       <c r="F244" s="5"/>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A245" s="3"/>
       <c r="B245" s="7" t="s">
         <v>629</v>
@@ -7085,7 +7091,7 @@
       <c r="E245" s="5"/>
       <c r="F245" s="5"/>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A246" s="3"/>
       <c r="B246" s="7" t="s">
         <v>632</v>
@@ -7099,7 +7105,7 @@
       <c r="E246" s="5"/>
       <c r="F246" s="5"/>
     </row>
-    <row r="247" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A247" s="3"/>
       <c r="B247" s="7" t="s">
         <v>635</v>
@@ -7113,7 +7119,7 @@
       <c r="E247" s="5"/>
       <c r="F247" s="5"/>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A248" s="3"/>
       <c r="B248" s="7" t="s">
         <v>638</v>
@@ -7127,7 +7133,7 @@
       <c r="E248" s="5"/>
       <c r="F248" s="5"/>
     </row>
-    <row r="249" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A249" s="3"/>
       <c r="B249" s="7" t="s">
         <v>641</v>
@@ -7141,7 +7147,7 @@
       <c r="E249" s="5"/>
       <c r="F249" s="5"/>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A250" s="3"/>
       <c r="B250" s="7" t="s">
         <v>644</v>
@@ -7155,7 +7161,7 @@
       <c r="E250" s="5"/>
       <c r="F250" s="5"/>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A251" s="3"/>
       <c r="B251" s="7" t="s">
         <v>647</v>
@@ -7169,7 +7175,7 @@
       <c r="E251" s="5"/>
       <c r="F251" s="5"/>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A252" s="3"/>
       <c r="B252" s="7" t="s">
         <v>650</v>
@@ -7183,7 +7189,7 @@
       <c r="E252" s="5"/>
       <c r="F252" s="5"/>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A253" s="3"/>
       <c r="B253" s="7" t="s">
         <v>653</v>
@@ -7197,7 +7203,7 @@
       <c r="E253" s="5"/>
       <c r="F253" s="5"/>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A254" s="3"/>
       <c r="B254" s="7" t="s">
         <v>656</v>
@@ -7211,7 +7217,7 @@
       <c r="E254" s="5"/>
       <c r="F254" s="5"/>
     </row>
-    <row r="255" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A255" s="3"/>
       <c r="B255" s="7" t="s">
         <v>659</v>
@@ -7227,7 +7233,7 @@
       </c>
       <c r="F255" s="5"/>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A256" s="3"/>
       <c r="B256" s="7" t="s">
         <v>662</v>
@@ -7241,7 +7247,7 @@
       <c r="E256" s="5"/>
       <c r="F256" s="5"/>
     </row>
-    <row r="257" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A257" s="3"/>
       <c r="B257" s="7" t="s">
         <v>665</v>
@@ -7255,7 +7261,7 @@
       <c r="E257" s="5"/>
       <c r="F257" s="5"/>
     </row>
-    <row r="258" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A258" s="3"/>
       <c r="B258" s="7" t="s">
         <v>668</v>
@@ -7271,7 +7277,7 @@
       </c>
       <c r="F258" s="5"/>
     </row>
-    <row r="259" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A259" s="3"/>
       <c r="B259" s="7" t="s">
         <v>671</v>
@@ -7287,7 +7293,7 @@
       </c>
       <c r="F259" s="5"/>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A260" s="3"/>
       <c r="B260" s="7" t="s">
         <v>674</v>
@@ -7301,7 +7307,7 @@
       <c r="E260" s="5"/>
       <c r="F260" s="5"/>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A261" s="3"/>
       <c r="B261" s="7" t="s">
         <v>677</v>
@@ -7315,7 +7321,7 @@
       <c r="E261" s="5"/>
       <c r="F261" s="5"/>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A262" s="3"/>
       <c r="B262" s="7" t="s">
         <v>680</v>
@@ -7329,7 +7335,7 @@
       <c r="E262" s="5"/>
       <c r="F262" s="5"/>
     </row>
-    <row r="263" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A263" s="3"/>
       <c r="B263" s="7" t="s">
         <v>683</v>
@@ -7343,7 +7349,7 @@
       <c r="E263" s="5"/>
       <c r="F263" s="5"/>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A264" s="3"/>
       <c r="B264" s="7" t="s">
         <v>686</v>
@@ -7357,7 +7363,7 @@
       <c r="E264" s="5"/>
       <c r="F264" s="5"/>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A265" s="3"/>
       <c r="B265" s="7" t="s">
         <v>689</v>
@@ -7371,7 +7377,7 @@
       <c r="E265" s="5"/>
       <c r="F265" s="5"/>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A266" s="3"/>
       <c r="B266" s="7" t="s">
         <v>692</v>
@@ -7385,7 +7391,7 @@
       <c r="E266" s="5"/>
       <c r="F266" s="5"/>
     </row>
-    <row r="267" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A267" s="3"/>
       <c r="B267" s="7" t="s">
         <v>695</v>
@@ -7399,7 +7405,7 @@
       <c r="E267" s="5"/>
       <c r="F267" s="5"/>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A268" s="3" t="s">
         <v>698</v>
       </c>
@@ -7409,7 +7415,7 @@
       <c r="E268" s="5"/>
       <c r="F268" s="5"/>
     </row>
-    <row r="269" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A269" s="3"/>
       <c r="B269" s="7" t="s">
         <v>699</v>
@@ -7423,7 +7429,7 @@
       <c r="E269" s="5"/>
       <c r="F269" s="5"/>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A270" s="3"/>
       <c r="B270" s="7" t="s">
         <v>702</v>
@@ -7437,7 +7443,7 @@
       <c r="E270" s="5"/>
       <c r="F270" s="5"/>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A271" s="3"/>
       <c r="B271" s="7" t="s">
         <v>705</v>
@@ -7451,7 +7457,7 @@
       <c r="E271" s="5"/>
       <c r="F271" s="5"/>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A272" s="3"/>
       <c r="B272" s="7" t="s">
         <v>708</v>
@@ -7465,7 +7471,7 @@
       <c r="E272" s="5"/>
       <c r="F272" s="5"/>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A273" s="3"/>
       <c r="B273" s="7" t="s">
         <v>711</v>
@@ -7479,7 +7485,7 @@
       <c r="E273" s="5"/>
       <c r="F273" s="5"/>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A274" s="3"/>
       <c r="B274" s="7" t="s">
         <v>714</v>
@@ -7493,7 +7499,7 @@
       <c r="E274" s="5"/>
       <c r="F274" s="5"/>
     </row>
-    <row r="275" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A275" s="3"/>
       <c r="B275" s="7" t="s">
         <v>717</v>
@@ -7507,7 +7513,7 @@
       <c r="E275" s="5"/>
       <c r="F275" s="5"/>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A276" s="3" t="s">
         <v>720</v>
       </c>
@@ -7517,7 +7523,7 @@
       <c r="E276" s="5"/>
       <c r="F276" s="5"/>
     </row>
-    <row r="277" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A277" s="3"/>
       <c r="B277" s="7" t="s">
         <v>721</v>
@@ -7533,7 +7539,7 @@
       </c>
       <c r="F277" s="5"/>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A278" s="3" t="s">
         <v>724</v>
       </c>
@@ -7543,7 +7549,7 @@
       <c r="E278" s="5"/>
       <c r="F278" s="5"/>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A279" s="3"/>
       <c r="B279" s="7" t="s">
         <v>725</v>
@@ -7557,7 +7563,7 @@
       <c r="E279" s="5"/>
       <c r="F279" s="5"/>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A280" s="3"/>
       <c r="B280" s="7" t="s">
         <v>728</v>
@@ -7571,7 +7577,7 @@
       <c r="E280" s="5"/>
       <c r="F280" s="5"/>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A281" s="3"/>
       <c r="B281" s="7" t="s">
         <v>731</v>
@@ -7585,7 +7591,7 @@
       <c r="E281" s="5"/>
       <c r="F281" s="5"/>
     </row>
-    <row r="282" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A282" s="3"/>
       <c r="B282" s="7" t="s">
         <v>734</v>
@@ -7599,7 +7605,7 @@
       <c r="E282" s="5"/>
       <c r="F282" s="5"/>
     </row>
-    <row r="283" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A283" s="3"/>
       <c r="B283" s="7" t="s">
         <v>737</v>
@@ -7615,7 +7621,7 @@
       </c>
       <c r="F283" s="5"/>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A284" s="3"/>
       <c r="B284" s="7" t="s">
         <v>740</v>
@@ -7629,7 +7635,7 @@
       <c r="E284" s="5"/>
       <c r="F284" s="5"/>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A285" s="3" t="s">
         <v>743</v>
       </c>
@@ -7639,7 +7645,7 @@
       <c r="E285" s="5"/>
       <c r="F285" s="5"/>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A286" s="3"/>
       <c r="B286" s="7" t="s">
         <v>744</v>
@@ -7653,7 +7659,7 @@
       <c r="E286" s="5"/>
       <c r="F286" s="5"/>
     </row>
-    <row r="287" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A287" s="3"/>
       <c r="B287" s="7" t="s">
         <v>747</v>
@@ -7667,7 +7673,7 @@
       <c r="E287" s="5"/>
       <c r="F287" s="5"/>
     </row>
-    <row r="288" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A288" s="3"/>
       <c r="B288" s="7" t="s">
         <v>750</v>
@@ -7683,7 +7689,7 @@
       </c>
       <c r="F288" s="5"/>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A289" s="3" t="s">
         <v>753</v>
       </c>
@@ -7693,7 +7699,7 @@
       <c r="E289" s="5"/>
       <c r="F289" s="5"/>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A290" s="3"/>
       <c r="B290" s="7" t="s">
         <v>754</v>
@@ -7707,7 +7713,7 @@
       <c r="E290" s="5"/>
       <c r="F290" s="5"/>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A291" s="3"/>
       <c r="B291" s="7" t="s">
         <v>754</v>
@@ -7721,7 +7727,7 @@
       <c r="E291" s="5"/>
       <c r="F291" s="5"/>
     </row>
-    <row r="292" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A292" s="3"/>
       <c r="B292" s="7" t="s">
         <v>757</v>
@@ -7735,7 +7741,7 @@
       <c r="E292" s="5"/>
       <c r="F292" s="5"/>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A293" s="3"/>
       <c r="B293" s="7" t="s">
         <v>760</v>
@@ -7749,7 +7755,7 @@
       <c r="E293" s="5"/>
       <c r="F293" s="5"/>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A294" s="3"/>
       <c r="B294" s="7" t="s">
         <v>763</v>
@@ -7763,7 +7769,7 @@
       <c r="E294" s="5"/>
       <c r="F294" s="5"/>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A295" s="3"/>
       <c r="B295" s="7" t="s">
         <v>766</v>
@@ -7777,7 +7783,7 @@
       <c r="E295" s="5"/>
       <c r="F295" s="5"/>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A296" s="3" t="s">
         <v>769</v>
       </c>
@@ -7787,7 +7793,7 @@
       <c r="E296" s="5"/>
       <c r="F296" s="5"/>
     </row>
-    <row r="297" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A297" s="3"/>
       <c r="B297" s="7" t="s">
         <v>770</v>
@@ -7801,7 +7807,7 @@
       <c r="E297" s="5"/>
       <c r="F297" s="5"/>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A298" s="3"/>
       <c r="B298" s="7" t="s">
         <v>773</v>
@@ -7815,7 +7821,7 @@
       <c r="E298" s="5"/>
       <c r="F298" s="5"/>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A299" s="3"/>
       <c r="B299" s="7" t="s">
         <v>776</v>
@@ -7829,7 +7835,7 @@
       <c r="E299" s="5"/>
       <c r="F299" s="5"/>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A300" s="3"/>
       <c r="B300" s="7" t="s">
         <v>779</v>
@@ -7843,7 +7849,7 @@
       <c r="E300" s="5"/>
       <c r="F300" s="5"/>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A301" s="3" t="s">
         <v>782</v>
       </c>
@@ -7853,7 +7859,7 @@
       <c r="E301" s="5"/>
       <c r="F301" s="5"/>
     </row>
-    <row r="302" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A302" s="3"/>
       <c r="B302" s="7" t="s">
         <v>783</v>
@@ -7867,7 +7873,7 @@
       <c r="E302" s="5"/>
       <c r="F302" s="5"/>
     </row>
-    <row r="303" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A303" s="3"/>
       <c r="B303" s="7" t="s">
         <v>786</v>
@@ -7881,7 +7887,7 @@
       <c r="E303" s="5"/>
       <c r="F303" s="5"/>
     </row>
-    <row r="304" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A304" s="3"/>
       <c r="B304" s="7" t="s">
         <v>789</v>
@@ -7895,7 +7901,7 @@
       <c r="E304" s="5"/>
       <c r="F304" s="5"/>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A305" s="3" t="s">
         <v>792</v>
       </c>
@@ -7905,7 +7911,7 @@
       <c r="E305" s="5"/>
       <c r="F305" s="5"/>
     </row>
-    <row r="306" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A306" s="3"/>
       <c r="B306" s="7" t="s">
         <v>793</v>
@@ -7919,7 +7925,7 @@
       <c r="E306" s="5"/>
       <c r="F306" s="5"/>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A307" s="3"/>
       <c r="B307" s="7" t="s">
         <v>796</v>
@@ -7933,7 +7939,7 @@
       <c r="E307" s="5"/>
       <c r="F307" s="5"/>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A308" s="3"/>
       <c r="B308" s="7" t="s">
         <v>799</v>
@@ -7947,7 +7953,7 @@
       <c r="E308" s="5"/>
       <c r="F308" s="5"/>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A309" s="3" t="s">
         <v>802</v>
       </c>
@@ -7957,7 +7963,7 @@
       <c r="E309" s="5"/>
       <c r="F309" s="5"/>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A310" s="3"/>
       <c r="B310" s="7" t="s">
         <v>803</v>
@@ -7971,7 +7977,7 @@
       <c r="E310" s="5"/>
       <c r="F310" s="5"/>
     </row>
-    <row r="311" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A311" s="3"/>
       <c r="B311" s="7" t="s">
         <v>806</v>
@@ -7985,7 +7991,7 @@
       <c r="E311" s="5"/>
       <c r="F311" s="5"/>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A312" s="3"/>
       <c r="B312" s="7" t="s">
         <v>809</v>
@@ -7999,7 +8005,7 @@
       <c r="E312" s="5"/>
       <c r="F312" s="5"/>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A313" s="3"/>
       <c r="B313" s="7" t="s">
         <v>812</v>
@@ -8013,7 +8019,7 @@
       <c r="E313" s="5"/>
       <c r="F313" s="5"/>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A314" s="3"/>
       <c r="B314" s="7" t="s">
         <v>815</v>
@@ -8027,7 +8033,7 @@
       <c r="E314" s="5"/>
       <c r="F314" s="5"/>
     </row>
-    <row r="315" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A315" s="3"/>
       <c r="B315" s="7" t="s">
         <v>818</v>
@@ -8041,7 +8047,7 @@
       <c r="E315" s="5"/>
       <c r="F315" s="5"/>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A316" s="3"/>
       <c r="B316" s="7" t="s">
         <v>821</v>
@@ -8055,7 +8061,7 @@
       <c r="E316" s="5"/>
       <c r="F316" s="5"/>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A317" s="3"/>
       <c r="B317" s="7" t="s">
         <v>824</v>
@@ -8069,7 +8075,7 @@
       <c r="E317" s="5"/>
       <c r="F317" s="5"/>
     </row>
-    <row r="318" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A318" s="3"/>
       <c r="B318" s="7" t="s">
         <v>827</v>
@@ -8083,7 +8089,7 @@
       <c r="E318" s="5"/>
       <c r="F318" s="5"/>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A319" s="3"/>
       <c r="B319" s="7" t="s">
         <v>830</v>
@@ -8099,7 +8105,7 @@
       </c>
       <c r="F319" s="5"/>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A320" s="3"/>
       <c r="B320" s="7" t="s">
         <v>833</v>
@@ -8115,7 +8121,7 @@
       </c>
       <c r="F320" s="5"/>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A321" s="3" t="s">
         <v>836</v>
       </c>
@@ -8125,7 +8131,7 @@
       <c r="E321" s="5"/>
       <c r="F321" s="5"/>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A322" s="3"/>
       <c r="B322" s="7" t="s">
         <v>837</v>
@@ -8139,7 +8145,7 @@
       <c r="E322" s="5"/>
       <c r="F322" s="5"/>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A323" s="3"/>
       <c r="B323" s="7" t="s">
         <v>840</v>
@@ -8153,7 +8159,7 @@
       <c r="E323" s="5"/>
       <c r="F323" s="5"/>
     </row>
-    <row r="324" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A324" s="3"/>
       <c r="B324" s="7" t="s">
         <v>843</v>
@@ -8169,7 +8175,7 @@
       </c>
       <c r="F324" s="5"/>
     </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A325" s="3"/>
       <c r="B325" s="7" t="s">
         <v>846</v>
@@ -8183,7 +8189,7 @@
       <c r="E325" s="5"/>
       <c r="F325" s="5"/>
     </row>
-    <row r="326" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A326" s="3"/>
       <c r="B326" s="7" t="s">
         <v>849</v>
@@ -8197,7 +8203,7 @@
       <c r="E326" s="5"/>
       <c r="F326" s="5"/>
     </row>
-    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A327" s="3"/>
       <c r="B327" s="7" t="s">
         <v>852</v>
@@ -8211,7 +8217,7 @@
       <c r="E327" s="5"/>
       <c r="F327" s="5"/>
     </row>
-    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A328" s="3"/>
       <c r="B328" s="7" t="s">
         <v>855</v>
@@ -8225,7 +8231,7 @@
       <c r="E328" s="5"/>
       <c r="F328" s="5"/>
     </row>
-    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A329" s="3"/>
       <c r="B329" s="7" t="s">
         <v>858</v>
@@ -8239,7 +8245,7 @@
       <c r="E329" s="5"/>
       <c r="F329" s="5"/>
     </row>
-    <row r="330" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A330" s="3"/>
       <c r="B330" s="7" t="s">
         <v>861</v>
@@ -8253,7 +8259,7 @@
       <c r="E330" s="5"/>
       <c r="F330" s="5"/>
     </row>
-    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A331" s="3"/>
       <c r="B331" s="7" t="s">
         <v>864</v>
@@ -8267,7 +8273,7 @@
       <c r="E331" s="5"/>
       <c r="F331" s="5"/>
     </row>
-    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A332" s="3"/>
       <c r="B332" s="7" t="s">
         <v>867</v>
@@ -8281,7 +8287,7 @@
       <c r="E332" s="5"/>
       <c r="F332" s="5"/>
     </row>
-    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A333" s="3"/>
       <c r="B333" s="7" t="s">
         <v>870</v>
@@ -8295,7 +8301,7 @@
       <c r="E333" s="5"/>
       <c r="F333" s="5"/>
     </row>
-    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A334" s="3"/>
       <c r="B334" s="7" t="s">
         <v>873</v>
@@ -8309,7 +8315,7 @@
       <c r="E334" s="5"/>
       <c r="F334" s="5"/>
     </row>
-    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A335" s="3"/>
       <c r="B335" s="7" t="s">
         <v>876</v>
@@ -8323,7 +8329,7 @@
       <c r="E335" s="5"/>
       <c r="F335" s="5"/>
     </row>
-    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A336" s="3"/>
       <c r="B336" s="7" t="s">
         <v>879</v>
@@ -8339,7 +8345,7 @@
       </c>
       <c r="F336" s="5"/>
     </row>
-    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A337" s="3"/>
       <c r="B337" s="7" t="s">
         <v>882</v>
@@ -8353,7 +8359,7 @@
       <c r="E337" s="5"/>
       <c r="F337" s="5"/>
     </row>
-    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A338" s="3"/>
       <c r="B338" s="7" t="s">
         <v>885</v>
@@ -8367,7 +8373,7 @@
       <c r="E338" s="5"/>
       <c r="F338" s="5"/>
     </row>
-    <row r="339" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A339" s="3"/>
       <c r="B339" s="7" t="s">
         <v>888</v>
@@ -8381,7 +8387,7 @@
       <c r="E339" s="5"/>
       <c r="F339" s="5"/>
     </row>
-    <row r="340" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A340" s="3"/>
       <c r="B340" s="7" t="s">
         <v>891</v>
@@ -8395,7 +8401,7 @@
       <c r="E340" s="5"/>
       <c r="F340" s="5"/>
     </row>
-    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A341" s="3"/>
       <c r="B341" s="7" t="s">
         <v>894</v>
@@ -8409,7 +8415,7 @@
       <c r="E341" s="5"/>
       <c r="F341" s="5"/>
     </row>
-    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A342" s="3" t="s">
         <v>897</v>
       </c>
@@ -8419,7 +8425,7 @@
       <c r="E342" s="5"/>
       <c r="F342" s="5"/>
     </row>
-    <row r="343" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A343" s="3"/>
       <c r="B343" s="7" t="s">
         <v>898</v>
@@ -8433,7 +8439,7 @@
       <c r="E343" s="5"/>
       <c r="F343" s="5"/>
     </row>
-    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A344" s="3"/>
       <c r="B344" s="7" t="s">
         <v>901</v>
@@ -8447,7 +8453,7 @@
       <c r="E344" s="5"/>
       <c r="F344" s="5"/>
     </row>
-    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A345" s="3"/>
       <c r="B345" s="7" t="s">
         <v>904</v>
@@ -8461,7 +8467,7 @@
       <c r="E345" s="5"/>
       <c r="F345" s="5"/>
     </row>
-    <row r="346" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A346" s="3"/>
       <c r="B346" s="7" t="s">
         <v>907</v>
@@ -8475,7 +8481,7 @@
       <c r="E346" s="5"/>
       <c r="F346" s="5"/>
     </row>
-    <row r="347" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A347" s="3"/>
       <c r="B347" s="7" t="s">
         <v>910</v>
@@ -8489,7 +8495,7 @@
       <c r="E347" s="5"/>
       <c r="F347" s="5"/>
     </row>
-    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A348" s="3"/>
       <c r="B348" s="7" t="s">
         <v>913</v>
@@ -8503,7 +8509,7 @@
       <c r="E348" s="5"/>
       <c r="F348" s="5"/>
     </row>
-    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A349" s="3"/>
       <c r="B349" s="7" t="s">
         <v>916</v>
@@ -8517,7 +8523,7 @@
       <c r="E349" s="5"/>
       <c r="F349" s="5"/>
     </row>
-    <row r="350" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A350" s="3"/>
       <c r="B350" s="7" t="s">
         <v>919</v>
@@ -8531,7 +8537,7 @@
       <c r="E350" s="5"/>
       <c r="F350" s="5"/>
     </row>
-    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A351" s="3"/>
       <c r="B351" s="7" t="s">
         <v>922</v>
@@ -8545,7 +8551,7 @@
       <c r="E351" s="5"/>
       <c r="F351" s="5"/>
     </row>
-    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A352" s="3" t="s">
         <v>925</v>
       </c>
@@ -8555,7 +8561,7 @@
       <c r="E352" s="5"/>
       <c r="F352" s="5"/>
     </row>
-    <row r="353" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A353" s="3"/>
       <c r="B353" s="7" t="s">
         <v>926</v>
@@ -8569,7 +8575,7 @@
       <c r="E353" s="5"/>
       <c r="F353" s="5"/>
     </row>
-    <row r="354" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A354" s="3"/>
       <c r="B354" s="7" t="s">
         <v>929</v>
@@ -8583,7 +8589,7 @@
       <c r="E354" s="5"/>
       <c r="F354" s="5"/>
     </row>
-    <row r="355" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A355" s="3"/>
       <c r="B355" s="7" t="s">
         <v>932</v>
@@ -8597,7 +8603,7 @@
       <c r="E355" s="5"/>
       <c r="F355" s="5"/>
     </row>
-    <row r="356" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A356" s="3"/>
       <c r="B356" s="7" t="s">
         <v>935</v>
@@ -8611,7 +8617,7 @@
       <c r="E356" s="5"/>
       <c r="F356" s="5"/>
     </row>
-    <row r="357" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A357" s="3"/>
       <c r="B357" s="7" t="s">
         <v>938</v>
@@ -8625,12 +8631,12 @@
       <c r="E357" s="5"/>
       <c r="F357" s="5"/>
     </row>
-    <row r="358" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A358" s="1" t="s">
         <v>944</v>
       </c>
     </row>
-    <row r="359" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A359" s="3"/>
       <c r="B359" s="7"/>
       <c r="C359" s="6"/>
@@ -8638,7 +8644,7 @@
       <c r="E359" s="5"/>
       <c r="F359" s="5"/>
     </row>
-    <row r="360" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A360" s="3"/>
       <c r="B360" s="7"/>
       <c r="C360" s="6"/>
@@ -8646,7 +8652,7 @@
       <c r="E360" s="5"/>
       <c r="F360" s="5"/>
     </row>
-    <row r="361" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A361" s="3"/>
       <c r="B361" s="7"/>
       <c r="C361" s="6"/>
@@ -8654,7 +8660,7 @@
       <c r="E361" s="5"/>
       <c r="F361" s="5"/>
     </row>
-    <row r="362" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A362" s="3"/>
       <c r="B362" s="7"/>
       <c r="C362" s="6"/>
@@ -8662,7 +8668,7 @@
       <c r="E362" s="5"/>
       <c r="F362" s="5"/>
     </row>
-    <row r="363" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A363" s="3"/>
       <c r="B363" s="7"/>
       <c r="C363" s="6"/>

</xml_diff>